<commit_message>
feat: add self-contained HEART AI chatbot (replaces n8n dependency)
- Add /heart-ai page with premium dark-themed chat UI
- Add OpenAI function-calling workflow replicating n8n HEART-Workflow
- Parse local data files (MasterSheet, PredictionText, Tweets, SourceOfTruth)
- Add /api/heart-chat API route with conversation history
- Update landing page navigation with HEART AI link
- Install mammoth for .docx parsing
</commit_message>
<xml_diff>
--- a/data/HEART_Model_khurshidOGcleaned.xlsx
+++ b/data/HEART_Model_khurshidOGcleaned.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Personal\Working on It\Eco\finalproduct\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A33E526-3586-47D6-9E01-FAF3B9927C75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{113FCED7-5F8E-4E75-8D28-6FACFECAFA60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-86" yWindow="0" windowWidth="11143" windowHeight="13080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HEART" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="Metadata" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -1327,7 +1328,7 @@
     <col min="36" max="36" width="14.15234375" customWidth="1"/>
     <col min="37" max="37" width="15.3828125" customWidth="1"/>
     <col min="38" max="38" width="29.765625" customWidth="1"/>
-    <col min="39" max="39" width="34.84375" customWidth="1"/>
+    <col min="39" max="39" width="38.69140625" bestFit="1" customWidth="1"/>
     <col min="40" max="40" width="36.4609375" customWidth="1"/>
     <col min="41" max="41" width="24.23046875" customWidth="1"/>
     <col min="42" max="42" width="235.23046875" customWidth="1"/>
@@ -1659,7 +1660,7 @@
     </row>
     <row r="4" spans="1:42" ht="33.9">
       <c r="A4" s="26">
-        <f t="shared" ref="A4:A6" si="19">A3+1</f>
+        <f>A3+1</f>
         <v>2</v>
       </c>
       <c r="B4" s="27" t="s">
@@ -1801,7 +1802,7 @@
     </row>
     <row r="5" spans="1:42" ht="33.9">
       <c r="A5" s="26">
-        <f t="shared" si="19"/>
+        <f>A4+1</f>
         <v>3</v>
       </c>
       <c r="B5" s="27" t="s">
@@ -1943,7 +1944,7 @@
     </row>
     <row r="6" spans="1:42" ht="33.9">
       <c r="A6" s="26">
-        <f t="shared" si="19"/>
+        <f>A5+1</f>
         <v>4</v>
       </c>
       <c r="B6" s="27" t="s">
@@ -2226,7 +2227,7 @@
     </row>
     <row r="8" spans="1:42" ht="33.9">
       <c r="A8" s="26">
-        <f t="shared" ref="A8:A10" si="20">A7+1</f>
+        <f>A7+1</f>
         <v>6</v>
       </c>
       <c r="B8" s="27" t="s">
@@ -2368,7 +2369,7 @@
     </row>
     <row r="9" spans="1:42" ht="33.9">
       <c r="A9" s="26">
-        <f t="shared" si="20"/>
+        <f>A8+1</f>
         <v>7</v>
       </c>
       <c r="B9" s="27" t="s">
@@ -2510,7 +2511,7 @@
     </row>
     <row r="10" spans="1:42" ht="33.9">
       <c r="A10" s="26">
-        <f t="shared" si="20"/>
+        <f>A9+1</f>
         <v>8</v>
       </c>
       <c r="B10" s="27" t="s">
@@ -2793,7 +2794,7 @@
     </row>
     <row r="12" spans="1:42" ht="33.9">
       <c r="A12" s="26">
-        <f t="shared" ref="A12:A14" si="21">A11+1</f>
+        <f>A11+1</f>
         <v>10</v>
       </c>
       <c r="B12" s="27" t="s">
@@ -3082,7 +3083,7 @@
     </row>
     <row r="14" spans="1:42" ht="33.9">
       <c r="A14" s="26">
-        <f t="shared" si="21"/>
+        <f>A13+1</f>
         <v>12</v>
       </c>
       <c r="B14" s="27" t="s">
@@ -3365,7 +3366,7 @@
     </row>
     <row r="16" spans="1:42" ht="33.9">
       <c r="A16" s="26">
-        <f t="shared" ref="A16:A18" si="22">A15+1</f>
+        <f>A15+1</f>
         <v>14</v>
       </c>
       <c r="B16" s="27" t="s">
@@ -3507,7 +3508,7 @@
     </row>
     <row r="17" spans="1:42" ht="33.9">
       <c r="A17" s="26">
-        <f t="shared" si="22"/>
+        <f>A16+1</f>
         <v>15</v>
       </c>
       <c r="B17" s="27" t="s">
@@ -3649,7 +3650,7 @@
     </row>
     <row r="18" spans="1:42" ht="33.9">
       <c r="A18" s="26">
-        <f t="shared" si="22"/>
+        <f>A17+1</f>
         <v>16</v>
       </c>
       <c r="B18" s="27" t="s">
@@ -3932,7 +3933,7 @@
     </row>
     <row r="20" spans="1:42" ht="33.9">
       <c r="A20" s="26">
-        <f t="shared" ref="A20:A21" si="23">A19+1</f>
+        <f>A19+1</f>
         <v>18</v>
       </c>
       <c r="B20" s="27" t="s">
@@ -4074,7 +4075,7 @@
     </row>
     <row r="21" spans="1:42" ht="33.9">
       <c r="A21" s="26">
-        <f t="shared" si="23"/>
+        <f>A20+1</f>
         <v>19</v>
       </c>
       <c r="B21" s="27" t="s">
@@ -4358,7 +4359,7 @@
     </row>
     <row r="23" spans="1:42" ht="33.9">
       <c r="A23" s="26">
-        <f t="shared" ref="A23:A24" si="24">A22+1</f>
+        <f>A22+1</f>
         <v>21</v>
       </c>
       <c r="B23" s="27" t="s">
@@ -4372,7 +4373,7 @@
         <v>20</v>
       </c>
       <c r="F23" s="29">
-        <f t="shared" ref="F23:F24" si="25">D23/$C$2</f>
+        <f>D23/$C$2</f>
         <v>6.0066692515334374E-3</v>
       </c>
       <c r="G23" s="12"/>
@@ -4380,18 +4381,18 @@
         <v>46700000</v>
       </c>
       <c r="I23" s="30">
-        <f t="shared" ref="I23:I24" si="26">H23/$G$2</f>
+        <f>H23/$G$2</f>
         <v>5.7062561094819155E-3</v>
       </c>
       <c r="J23" s="31">
-        <f t="shared" ref="J23:J24" si="27">D23/H23</f>
+        <f>D23/H23</f>
         <v>14636.680942184154</v>
       </c>
       <c r="K23" s="30">
         <v>0.318</v>
       </c>
       <c r="L23" s="32">
-        <f t="shared" ref="L23:L24" si="28">J23-J23*K23</f>
+        <f>J23-J23*K23</f>
         <v>9982.2164025695929</v>
       </c>
       <c r="M23" s="30">
@@ -4405,15 +4406,15 @@
         <v>154744000000</v>
       </c>
       <c r="P23" s="14">
-        <f t="shared" ref="P23:P24" si="29">N23+O23</f>
+        <f>N23+O23</f>
         <v>688344000000</v>
       </c>
       <c r="Q23" s="29">
-        <f t="shared" ref="Q23:Q24" si="30">O23/D23</f>
+        <f>O23/D23</f>
         <v>0.22638848453549426</v>
       </c>
       <c r="R23" s="30">
-        <f t="shared" ref="R23:R24" si="31">P23/D23</f>
+        <f>P23/D23</f>
         <v>1.0070384312096123</v>
       </c>
       <c r="S23" s="12"/>
@@ -4421,57 +4422,57 @@
         <v>141000000000</v>
       </c>
       <c r="U23" s="30">
-        <f t="shared" ref="U23:U24" si="32">T23/$S$2</f>
+        <f>T23/$S$2</f>
         <v>2.2720314539389935E-3</v>
       </c>
       <c r="V23" s="30">
-        <f t="shared" ref="V23:V24" si="33">T23/D23</f>
+        <f>T23/D23</f>
         <v>0.20628118905744128</v>
       </c>
       <c r="W23" s="46">
         <v>19000000000</v>
       </c>
       <c r="X23" s="35">
-        <f t="shared" ref="X23:X24" si="34">W23/D23</f>
+        <f>W23/D23</f>
         <v>2.7796755972279319E-2</v>
       </c>
       <c r="Y23" s="14">
         <v>116200000000</v>
       </c>
       <c r="Z23" s="29">
-        <f t="shared" ref="Z23:Z24" si="35">Y23/D23</f>
+        <f>Y23/D23</f>
         <v>0.16999910757783457</v>
       </c>
       <c r="AA23" s="36">
         <v>14400000</v>
       </c>
       <c r="AB23" s="37">
-        <f t="shared" ref="AB23:AB24" si="36">AA23/H23</f>
+        <f>AA23/H23</f>
         <v>0.30835117773019272</v>
       </c>
       <c r="AC23" s="38">
         <v>68353000000</v>
       </c>
       <c r="AD23" s="29">
-        <f t="shared" ref="AD23:AD24" si="37">AC23/D23</f>
+        <f>AC23/D23</f>
         <v>9.9999561103853066E-2</v>
       </c>
       <c r="AE23" s="31">
         <v>54640000000</v>
       </c>
       <c r="AF23" s="29">
-        <f t="shared" ref="AF23:AF24" si="38">AE23/D23</f>
+        <f>AE23/D23</f>
         <v>7.9937618227649582E-2</v>
       </c>
       <c r="AG23" s="31">
         <v>41000000000</v>
       </c>
       <c r="AH23" s="29">
-        <f t="shared" ref="AH23:AH24" si="39">AG23/D23</f>
+        <f>AG23/D23</f>
         <v>5.9982473413865901E-2</v>
       </c>
       <c r="AI23" s="39">
-        <f t="shared" ref="AI23:AI24" si="40">(AH23+AF23+AD23+Z23+F23-Q23+X23)</f>
+        <f>(AH23+AF23+AD23+Z23+F23-Q23+X23)</f>
         <v>0.21733370101152155</v>
       </c>
       <c r="AJ23" s="40">
@@ -4481,11 +4482,11 @@
         <v>0.4</v>
       </c>
       <c r="AL23" s="41">
-        <f t="shared" ref="AL23:AL24" si="41">AJ23-AK23</f>
+        <f>AJ23-AK23</f>
         <v>0.46499999999999997</v>
       </c>
       <c r="AM23" s="42">
-        <f t="shared" ref="AM23:AM24" si="42">(L23)*(AL23)</f>
+        <f>(L23)*(AL23)</f>
         <v>4641.7306271948601</v>
       </c>
       <c r="AN23" s="43" t="s">
@@ -4500,7 +4501,7 @@
     </row>
     <row r="24" spans="1:42" ht="33.9">
       <c r="A24" s="26">
-        <f t="shared" si="24"/>
+        <f>A23+1</f>
         <v>22</v>
       </c>
       <c r="B24" s="27" t="s">
@@ -4514,7 +4515,7 @@
         <v>38</v>
       </c>
       <c r="F24" s="29">
-        <f t="shared" si="25"/>
+        <f>D24/$C$2</f>
         <v>3.7468909847349387E-3</v>
       </c>
       <c r="G24" s="12"/>
@@ -4522,18 +4523,18 @@
         <v>64010000</v>
       </c>
       <c r="I24" s="30">
-        <f t="shared" si="26"/>
+        <f>H24/$G$2</f>
         <v>7.8213587487781042E-3</v>
       </c>
       <c r="J24" s="31">
-        <f t="shared" si="27"/>
+        <f>D24/H24</f>
         <v>6661.1466958287765</v>
       </c>
       <c r="K24" s="30">
         <v>3.4000000000000002E-2</v>
       </c>
       <c r="L24" s="32">
-        <f t="shared" si="28"/>
+        <f>J24-J24*K24</f>
         <v>6434.6677081705984</v>
       </c>
       <c r="M24" s="30">
@@ -4543,19 +4544,19 @@
         <v>332576000000</v>
       </c>
       <c r="O24" s="14">
-        <f t="shared" ref="O24" si="43">N24*M24</f>
+        <f>N24*M24</f>
         <v>22448880000</v>
       </c>
       <c r="P24" s="14">
-        <f t="shared" si="29"/>
+        <f>N24+O24</f>
         <v>355024880000</v>
       </c>
       <c r="Q24" s="29">
-        <f t="shared" si="30"/>
+        <f>O24/D24</f>
         <v>5.2649936676204323E-2</v>
       </c>
       <c r="R24" s="30">
-        <f t="shared" si="31"/>
+        <f>P24/D24</f>
         <v>0.83264899854589802</v>
       </c>
       <c r="S24" s="12"/>
@@ -4563,57 +4564,57 @@
         <v>252000000000</v>
       </c>
       <c r="U24" s="30">
-        <f t="shared" si="32"/>
+        <f>T24/$S$2</f>
         <v>4.0606519602313929E-3</v>
       </c>
       <c r="V24" s="30">
-        <f t="shared" si="33"/>
+        <f>T24/D24</f>
         <v>0.59102209296871333</v>
       </c>
       <c r="W24" s="46">
         <v>38000000000</v>
       </c>
       <c r="X24" s="35">
-        <f t="shared" si="34"/>
+        <f>W24/D24</f>
         <v>8.9122379098456772E-2</v>
       </c>
       <c r="Y24" s="14">
         <v>65803000000</v>
       </c>
       <c r="Z24" s="29">
-        <f t="shared" si="35"/>
+        <f>Y24/D24</f>
         <v>0.15432947136357239</v>
       </c>
       <c r="AA24" s="36">
         <v>20000000</v>
       </c>
       <c r="AB24" s="37">
-        <f t="shared" si="36"/>
+        <f>AA24/H24</f>
         <v>0.31245117950320261</v>
       </c>
       <c r="AC24" s="38">
         <v>36374000000</v>
       </c>
       <c r="AD24" s="29">
-        <f t="shared" si="37"/>
+        <f>AC24/D24</f>
         <v>8.5308879403349122E-2</v>
       </c>
       <c r="AE24" s="31">
         <v>25582000000</v>
       </c>
       <c r="AF24" s="29">
-        <f t="shared" si="38"/>
+        <f>AE24/D24</f>
         <v>5.9998123739387399E-2</v>
       </c>
       <c r="AG24" s="31">
         <v>27714000000</v>
       </c>
       <c r="AH24" s="29">
-        <f t="shared" si="39"/>
+        <f>AG24/D24</f>
         <v>6.4998358271963971E-2</v>
       </c>
       <c r="AI24" s="39">
-        <f t="shared" si="40"/>
+        <f>(AH24+AF24+AD24+Z24+F24-Q24+X24)</f>
         <v>0.40485416618526032</v>
       </c>
       <c r="AJ24" s="40">
@@ -4623,11 +4624,11 @@
         <v>0.63</v>
       </c>
       <c r="AL24" s="41">
-        <f t="shared" si="41"/>
+        <f>AJ24-AK24</f>
         <v>0.10999999999999999</v>
       </c>
       <c r="AM24" s="42">
-        <f t="shared" si="42"/>
+        <f>(L24)*(AL24)</f>
         <v>707.81344789876573</v>
       </c>
       <c r="AN24" s="43" t="s">

</xml_diff>